<commit_message>
Added examplary input, config, and sequence files
</commit_message>
<xml_diff>
--- a/af3_input.xlsx
+++ b/af3_input.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jan\projects\github\af3-server-workflow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC5F03C7-79A3-4A06-BDDD-3C9F9EF46CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAED7C2B-C0C7-47E9-B99A-E2C503D12FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DF82DD98-647C-46FD-B2CB-3DA0B17EFD46}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{DF82DD98-647C-46FD-B2CB-3DA0B17EFD46}"/>
   </bookViews>
   <sheets>
-    <sheet name="0001_20260101_0Ca1AtM21CAM2" sheetId="137" r:id="rId1"/>
-    <sheet name="0001_20260101_0Ca1AtM2LWRR1CAM2" sheetId="138" r:id="rId2"/>
-    <sheet name="0001_20260101_4Ca1AtM21CAM2" sheetId="139" r:id="rId3"/>
-    <sheet name="0001_20260101_4Ca1AtM2LWRR1CAM2" sheetId="140" r:id="rId4"/>
+    <sheet name="0001_20260101_AtMLO1AtCAM2" sheetId="142" r:id="rId1"/>
+    <sheet name="0002_20260101_AtMLO2AtCAM2" sheetId="141" r:id="rId2"/>
+    <sheet name="0003_20260101_0Ca1AtM21CAM2" sheetId="137" r:id="rId3"/>
+    <sheet name="0004_20260101_0Ca1AtM2LWRR1CAM2" sheetId="138" r:id="rId4"/>
+    <sheet name="0005_20260101_4Ca1AtM21CAM2" sheetId="139" r:id="rId5"/>
+    <sheet name="0006_20260101_4Ca1AtM2LWRR1CAM2" sheetId="140" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="52">
   <si>
     <t>AtMLO2.1CT</t>
   </si>
@@ -179,16 +181,25 @@
     <t>AtCAM2.1</t>
   </si>
   <si>
-    <t>0132</t>
-  </si>
-  <si>
-    <t>0133</t>
-  </si>
-  <si>
-    <t>0134</t>
-  </si>
-  <si>
-    <t>0135</t>
+    <t>AtMLO2.1</t>
+  </si>
+  <si>
+    <t>0002</t>
+  </si>
+  <si>
+    <t>AtMLO1.1</t>
+  </si>
+  <si>
+    <t>0003</t>
+  </si>
+  <si>
+    <t>0004</t>
+  </si>
+  <si>
+    <t>0005</t>
+  </si>
+  <si>
+    <t>0006</t>
   </si>
 </sst>
 </file>
@@ -577,6 +588,1274 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6C89F2A-14B5-41E8-89A3-3E8129747581}">
+  <sheetPr>
+    <tabColor theme="5"/>
+  </sheetPr>
+  <dimension ref="A1:R21"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="44" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="45.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O1" t="s">
+        <v>24</v>
+      </c>
+      <c r="P1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>_xlfn.CONCAT(B2,"-",C2,"-",D2,"_",F2,E2,"_",G2,SUBSTITUTE(I2,".1",""),J2,SUBSTITUTE(L2,".1",""),M2,SUBSTITUTE(O2,".1",""),P2,SUBSTITUTE(R2,".1",""))</f>
+        <v>0002-01-1710_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="str">
+        <f>HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; I2 &amp; ".fasta", "sequences\" &amp; I2 &amp; ".fasta")</f>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="str">
+        <f>HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; L2 &amp; ".fasta", "sequences\" &amp; L2 &amp; ".fasta")</f>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" s="2"/>
+      <c r="Q2" s="2"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f t="shared" ref="A3:A13" si="0">_xlfn.CONCAT(B3,"-",C3,"-",D3,"_",F3,E3,"_",G3,SUBSTITUTE(I3,".1",""),J3,SUBSTITUTE(L3,".1",""),M3,SUBSTITUTE(O3,".1",""),P3,SUBSTITUTE(R3,".1",""))</f>
+        <v>0002-02-1711_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="str">
+        <f t="shared" ref="H3:H13" si="1">HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; I3 &amp; ".fasta", "sequences\" &amp; I3 &amp; ".fasta")</f>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="str">
+        <f t="shared" ref="K3:K13" si="2">HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; L3 &amp; ".fasta", "sequences\" &amp; L3 &amp; ".fasta")</f>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L3" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q3" s="2"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-03-1712_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I4" t="s">
+        <v>47</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L4" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q4" s="2"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-04-1701_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I5" t="s">
+        <v>47</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L5" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q5" s="2"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-05-1702_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I6" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q6" s="2"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-06-1703_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I7" t="s">
+        <v>47</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L7" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q7" s="2"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-07-1704_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I8" t="s">
+        <v>47</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-08-1705_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I9" t="s">
+        <v>47</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-09-1706_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10">
+        <v>4</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-10-1707_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I11" t="s">
+        <v>47</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-11-1708_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12">
+        <v>4</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I12" t="s">
+        <v>47</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-12-1709_4CA_1AtMLO11AtCAM2</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO1.1.fasta</v>
+      </c>
+      <c r="I13" t="s">
+        <v>47</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="H21" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{737E6D8E-2329-4CF6-A84A-8CDF7B401001}">
+  <sheetPr>
+    <tabColor theme="5"/>
+  </sheetPr>
+  <dimension ref="A1:R21"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="44" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="45.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" t="s">
+        <v>21</v>
+      </c>
+      <c r="L1" t="s">
+        <v>22</v>
+      </c>
+      <c r="M1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O1" t="s">
+        <v>24</v>
+      </c>
+      <c r="P1" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>_xlfn.CONCAT(B2,"-",C2,"-",D2,"_",F2,E2,"_",G2,SUBSTITUTE(I2,".1",""),J2,SUBSTITUTE(L2,".1",""),M2,SUBSTITUTE(O2,".1",""),P2,SUBSTITUTE(R2,".1",""))</f>
+        <v>0002-01-1710_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="str">
+        <f>HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; I2 &amp; ".fasta", "sequences\" &amp; I2 &amp; ".fasta")</f>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="str">
+        <f>HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; L2 &amp; ".fasta", "sequences\" &amp; L2 &amp; ".fasta")</f>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" s="2"/>
+      <c r="Q2" s="2"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f t="shared" ref="A3:A13" si="0">_xlfn.CONCAT(B3,"-",C3,"-",D3,"_",F3,E3,"_",G3,SUBSTITUTE(I3,".1",""),J3,SUBSTITUTE(L3,".1",""),M3,SUBSTITUTE(O3,".1",""),P3,SUBSTITUTE(R3,".1",""))</f>
+        <v>0002-02-1711_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="str">
+        <f t="shared" ref="H3:H13" si="1">HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; I3 &amp; ".fasta", "sequences\" &amp; I3 &amp; ".fasta")</f>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I3" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="str">
+        <f t="shared" ref="K3:K13" si="2">HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; L3 &amp; ".fasta", "sequences\" &amp; L3 &amp; ".fasta")</f>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L3" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q3" s="2"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-03-1712_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L4" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q4" s="2"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-04-1701_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L5" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q5" s="2"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-05-1702_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I6" t="s">
+        <v>45</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q6" s="2"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-06-1703_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L7" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q7" s="2"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-07-1704_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I8" t="s">
+        <v>45</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-08-1705_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I9" t="s">
+        <v>45</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-09-1706_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10">
+        <v>4</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I10" t="s">
+        <v>45</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-10-1707_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I11" t="s">
+        <v>45</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-11-1708_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12">
+        <v>4</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I12" t="s">
+        <v>45</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <f t="shared" si="0"/>
+        <v>0002-12-1709_4CA_1AtMLO21AtCAM2</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>sequences\AtMLO2.1.fasta</v>
+      </c>
+      <c r="I13" t="s">
+        <v>45</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>sequences\AtCAM2.1.fasta</v>
+      </c>
+      <c r="L13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="H21" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA8D3B2D-9C74-4FFD-B67C-3A4E5A1B4050}">
   <sheetPr>
     <tabColor theme="5"/>
@@ -659,10 +1938,10 @@
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>_xlfn.CONCAT(B2,"-",C2,"-",D2,"_",F2,E2,"_",G2,SUBSTITUTE(I2,".1",""),J2,SUBSTITUTE(L2,".1",""),M2,SUBSTITUTE(O2,".1",""),P2,SUBSTITUTE(R2,".1",""))</f>
-        <v>0132-01-1710_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-01-1710_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>5</v>
@@ -702,10 +1981,10 @@
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f t="shared" ref="A3:A13" si="0">_xlfn.CONCAT(B3,"-",C3,"-",D3,"_",F3,E3,"_",G3,SUBSTITUTE(I3,".1",""),J3,SUBSTITUTE(L3,".1",""),M3,SUBSTITUTE(O3,".1",""),P3,SUBSTITUTE(R3,".1",""))</f>
-        <v>0132-02-1711_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-02-1711_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -744,10 +2023,10 @@
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
-        <v>0132-03-1712_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-03-1712_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -786,10 +2065,10 @@
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
-        <v>0132-04-1701_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-04-1701_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>8</v>
@@ -828,10 +2107,10 @@
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
-        <v>0132-05-1702_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-05-1702_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>9</v>
@@ -870,10 +2149,10 @@
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
-        <v>0132-06-1703_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-06-1703_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>10</v>
@@ -912,10 +2191,10 @@
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
-        <v>0132-07-1704_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-07-1704_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>11</v>
@@ -953,10 +2232,10 @@
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
-        <v>0132-08-1705_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-08-1705_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>12</v>
@@ -994,10 +2273,10 @@
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
-        <v>0132-09-1706_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-09-1706_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>13</v>
@@ -1035,10 +2314,10 @@
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
-        <v>0132-10-1707_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-10-1707_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>14</v>
@@ -1076,10 +2355,10 @@
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
-        <v>0132-11-1708_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-11-1708_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>15</v>
@@ -1117,10 +2396,10 @@
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
-        <v>0132-12-1709_0Ions_1AtMLO2CT1AtCAM2</v>
+        <v>0003-12-1709_0Ions_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>16</v>
@@ -1210,7 +2489,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{150D7FBF-A2E6-4DE5-B932-695BE9C01E91}">
   <sheetPr>
     <tabColor theme="5"/>
@@ -1218,7 +2497,7 @@
   <dimension ref="A1:R21"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="50.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="3.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.140625" bestFit="1" customWidth="1"/>
@@ -1293,10 +2572,10 @@
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>_xlfn.CONCAT(B2,"-",C2,"-",D2,"_",F2,E2,"_",G2,SUBSTITUTE(I2,".1",""),J2,SUBSTITUTE(L2,".1",""),M2,SUBSTITUTE(O2,".1",""),P2,SUBSTITUTE(R2,".1",""))</f>
-        <v>0133-01-1710_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-01-1710_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>5</v>
@@ -1336,10 +2615,10 @@
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f t="shared" ref="A3:A13" si="0">_xlfn.CONCAT(B3,"-",C3,"-",D3,"_",F3,E3,"_",G3,SUBSTITUTE(I3,".1",""),J3,SUBSTITUTE(L3,".1",""),M3,SUBSTITUTE(O3,".1",""),P3,SUBSTITUTE(R3,".1",""))</f>
-        <v>0133-02-1711_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-02-1711_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -1378,10 +2657,10 @@
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
-        <v>0133-03-1712_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-03-1712_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -1420,10 +2699,10 @@
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
-        <v>0133-04-1701_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-04-1701_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>8</v>
@@ -1462,10 +2741,10 @@
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
-        <v>0133-05-1702_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-05-1702_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>9</v>
@@ -1504,10 +2783,10 @@
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
-        <v>0133-06-1703_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-06-1703_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>10</v>
@@ -1546,10 +2825,10 @@
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
-        <v>0133-07-1704_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-07-1704_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>11</v>
@@ -1587,10 +2866,10 @@
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
-        <v>0133-08-1705_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-08-1705_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>12</v>
@@ -1628,10 +2907,10 @@
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
-        <v>0133-09-1706_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-09-1706_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>13</v>
@@ -1669,10 +2948,10 @@
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
-        <v>0133-10-1707_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-10-1707_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>14</v>
@@ -1710,10 +2989,10 @@
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
-        <v>0133-11-1708_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-11-1708_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>15</v>
@@ -1751,10 +3030,10 @@
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
-        <v>0133-12-1709_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0004-12-1709_0Ions_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>16</v>
@@ -1844,7 +3123,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C046188-19DE-45D7-9B7D-9581D26676CF}">
   <sheetPr>
     <tabColor theme="5"/>
@@ -1927,10 +3206,10 @@
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>_xlfn.CONCAT(B2,"-",C2,"-",D2,"_",F2,E2,"_",G2,SUBSTITUTE(I2,".1",""),J2,SUBSTITUTE(L2,".1",""),M2,SUBSTITUTE(O2,".1",""),P2,SUBSTITUTE(R2,".1",""))</f>
-        <v>0134-01-1710_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-01-1710_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>5</v>
@@ -1970,10 +3249,10 @@
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f t="shared" ref="A3:A13" si="0">_xlfn.CONCAT(B3,"-",C3,"-",D3,"_",F3,E3,"_",G3,SUBSTITUTE(I3,".1",""),J3,SUBSTITUTE(L3,".1",""),M3,SUBSTITUTE(O3,".1",""),P3,SUBSTITUTE(R3,".1",""))</f>
-        <v>0134-02-1711_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-02-1711_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -2012,10 +3291,10 @@
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
-        <v>0134-03-1712_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-03-1712_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -2054,10 +3333,10 @@
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
-        <v>0134-04-1701_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-04-1701_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>8</v>
@@ -2096,10 +3375,10 @@
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
-        <v>0134-05-1702_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-05-1702_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>9</v>
@@ -2138,10 +3417,10 @@
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
-        <v>0134-06-1703_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-06-1703_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>10</v>
@@ -2180,10 +3459,10 @@
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
-        <v>0134-07-1704_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-07-1704_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>11</v>
@@ -2221,10 +3500,10 @@
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
-        <v>0134-08-1705_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-08-1705_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>12</v>
@@ -2262,10 +3541,10 @@
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
-        <v>0134-09-1706_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-09-1706_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>13</v>
@@ -2303,10 +3582,10 @@
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
-        <v>0134-10-1707_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-10-1707_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>14</v>
@@ -2344,10 +3623,10 @@
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
-        <v>0134-11-1708_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-11-1708_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>15</v>
@@ -2385,10 +3664,10 @@
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
-        <v>0134-12-1709_4CA_1AtMLO2CT1AtCAM2</v>
+        <v>0005-12-1709_4CA_1AtMLO2CT1AtCAM2</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>16</v>
@@ -2478,7 +3757,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF592D66-CD80-45BE-B03B-D0EBBE136DC5}">
   <sheetPr>
     <tabColor theme="5"/>
@@ -2561,10 +3840,10 @@
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="str">
         <f>_xlfn.CONCAT(B2,"-",C2,"-",D2,"_",F2,E2,"_",G2,SUBSTITUTE(I2,".1",""),J2,SUBSTITUTE(L2,".1",""),M2,SUBSTITUTE(O2,".1",""),P2,SUBSTITUTE(R2,".1",""))</f>
-        <v>0135-01-1710_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-01-1710_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>5</v>
@@ -2604,10 +3883,10 @@
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f t="shared" ref="A3:A13" si="0">_xlfn.CONCAT(B3,"-",C3,"-",D3,"_",F3,E3,"_",G3,SUBSTITUTE(I3,".1",""),J3,SUBSTITUTE(L3,".1",""),M3,SUBSTITUTE(O3,".1",""),P3,SUBSTITUTE(R3,".1",""))</f>
-        <v>0135-02-1711_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-02-1711_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -2635,7 +3914,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="2" t="str">
-        <f t="shared" ref="K3:K14" si="2">HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; L3 &amp; ".fasta", "sequences\" &amp; L3 &amp; ".fasta")</f>
+        <f t="shared" ref="K3:K13" si="2">HYPERLINK("file://\\wsl.localhost\Ubuntu\home\user\projects\af3_workflow\sequences/" &amp; L3 &amp; ".fasta", "sequences\" &amp; L3 &amp; ".fasta")</f>
         <v>sequences\AtCAM2.1.fasta</v>
       </c>
       <c r="L3" t="s">
@@ -2646,10 +3925,10 @@
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
-        <v>0135-03-1712_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-03-1712_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -2688,10 +3967,10 @@
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
-        <v>0135-04-1701_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-04-1701_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>8</v>
@@ -2730,10 +4009,10 @@
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
-        <v>0135-05-1702_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-05-1702_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>9</v>
@@ -2772,10 +4051,10 @@
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
-        <v>0135-06-1703_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-06-1703_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>10</v>
@@ -2814,10 +4093,10 @@
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
-        <v>0135-07-1704_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-07-1704_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>11</v>
@@ -2855,10 +4134,10 @@
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
-        <v>0135-08-1705_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-08-1705_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>12</v>
@@ -2896,10 +4175,10 @@
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
-        <v>0135-09-1706_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-09-1706_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>13</v>
@@ -2937,10 +4216,10 @@
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
         <f t="shared" si="0"/>
-        <v>0135-10-1707_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-10-1707_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>14</v>
@@ -2978,10 +4257,10 @@
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
         <f t="shared" si="0"/>
-        <v>0135-11-1708_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-11-1708_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>15</v>
@@ -3019,10 +4298,10 @@
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
         <f t="shared" si="0"/>
-        <v>0135-12-1709_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
+        <v>0006-12-1709_4CA_1AtMLO2CT_L456R_W459R1AtCAM2</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>16</v>

</xml_diff>